<commit_message>
EXCEL LC AUTO changes
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/data inputs/Product-Description-inputs-Jeans.xlsx
+++ b/Full-LC-AUTO/data inputs/Product-Description-inputs-Jeans.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work-mom\Code-Tools\Full-LC-AUTO\data inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESHAAN\HAKUR\work--fk-tools\Full-LC-AUTO\data inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159941D3-0F9E-46A4-8758-3BA4B45BC9FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8B626B-D82C-4A84-8858-022B69072F9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="51">
   <si>
     <t>kind</t>
   </si>
@@ -162,6 +162,18 @@
   </si>
   <si>
     <t>BEG-NY-</t>
+  </si>
+  <si>
+    <t>ICE-NY-</t>
+  </si>
+  <si>
+    <t>BBP-NY-</t>
+  </si>
+  <si>
+    <t>BPJ-NY-</t>
+  </si>
+  <si>
+    <t>WPJ-NY-</t>
   </si>
 </sst>
 </file>
@@ -930,7 +942,7 @@
         <v>43</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>17</v>
@@ -980,7 +992,7 @@
         <v>43</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>17</v>
@@ -1030,7 +1042,7 @@
         <v>43</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>16</v>
@@ -1080,7 +1092,7 @@
         <v>43</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>16</v>

</xml_diff>